<commit_message>
🍏 Processed total 345 companies from Tier_1_BATCH_1561-2070 ( Found 1425 Contacts ) ✅
</commit_message>
<xml_diff>
--- a/OLD_OUTPUT/run_13may2026/apollo_people_search_13may2026_153853.xlsx
+++ b/OLD_OUTPUT/run_13may2026/apollo_people_search_13may2026_153853.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="160" documentId="11_A9E0AFFAB01C1A7CF102DC74305BDA16B6442522" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7BCEE7C-E5BB-4703-9B98-E38777B413EC}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="11_A9E0AFFAB01C1A7CF102DC74305BDA16B6442522" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91D0014C-D75D-4E7E-B505-BE52CCB415E6}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contacts" sheetId="1" r:id="rId1"/>

</xml_diff>